<commit_message>
update 1 from final review
</commit_message>
<xml_diff>
--- a/CostBreakdown.xlsx
+++ b/CostBreakdown.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jpreisle\Documents\Visual Studio\Git\451-DBF-Team01\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jpreisle\Documents\GitHub\451-DBF-Team01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{812E67BB-1D44-4D6D-9542-41B82AC33CDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30CE0B5A-9AC3-48EE-B041-D981C7776F01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="831" activeTab="5" xr2:uid="{C684E4FE-65D8-41BB-8319-3046AEA9131B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="831" activeTab="3" xr2:uid="{C684E4FE-65D8-41BB-8319-3046AEA9131B}"/>
   </bookViews>
   <sheets>
     <sheet name="Aircraft Cost Grand Total" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="97">
   <si>
     <t>M4 30mm bolt</t>
   </si>
@@ -64,12 +64,6 @@
     <t>Link</t>
   </si>
   <si>
-    <t>10x7E Prop</t>
-  </si>
-  <si>
-    <t>Cobra 3520/10</t>
-  </si>
-  <si>
     <t>RC Electric Parts 80A ESC</t>
   </si>
   <si>
@@ -130,9 +124,6 @@
     <t>https://www.homedepot.com/p/Owens-Corning-FOAMULAR-NGX-F-250-2-in-x-4-ft-x-8-ft-SSE-R-10-XPS-Rigid-Foam-Board-Insulation-52DDNGX/315197962</t>
   </si>
   <si>
-    <t>https://www.apcprop.com/product/10x7e/?v=0b3b97fa6688</t>
-  </si>
-  <si>
     <t>Purchased</t>
   </si>
   <si>
@@ -151,9 +142,6 @@
     <t>Propulsion</t>
   </si>
   <si>
-    <t>https://www.cobramotorsusa.com/motors-3520-10.html</t>
-  </si>
-  <si>
     <t>https://www.amazon.com/RC-Electric-Controller-Brushless-Motors/dp/B071GRSFBD?th=1</t>
   </si>
   <si>
@@ -295,21 +283,6 @@
     <t>Aluminum 40mm x 8 mm OD Spacer</t>
   </si>
   <si>
-    <t>3M Pads</t>
-  </si>
-  <si>
-    <t>change to PETG</t>
-  </si>
-  <si>
-    <t>find cost and verify quantity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">single sided velcro </t>
-  </si>
-  <si>
-    <t>Duct Tape</t>
-  </si>
-  <si>
     <t>Bambu Skewers</t>
   </si>
   <si>
@@ -319,10 +292,49 @@
     <t>maybe use easy connectors instead</t>
   </si>
   <si>
-    <t>check 3520/12</t>
-  </si>
-  <si>
-    <t>check 11x8E</t>
+    <t>11x85E Prop</t>
+  </si>
+  <si>
+    <t>Cobra 3520/12</t>
+  </si>
+  <si>
+    <t>https://www.cobramotorsusa.com/motors-3520-12.html</t>
+  </si>
+  <si>
+    <t>https://us.store.bambulab.com/products/petg-basic</t>
+  </si>
+  <si>
+    <t>https://www.horizonhobby.com/product/apc-landing-products-electric-propeller-11-x-8.5e/APC11085E.html</t>
+  </si>
+  <si>
+    <t>https://www.uline.com/Product/Detail/S-24954/3M-Double-Sided-Tape/3M-GPT-020-Double-Coated-Tape-1-2-x-55-yds?pricode=WB2129&amp;gadtype=pla&amp;id=S-24954&amp;ad_group_id=145971513970&amp;gad_source=1&amp;gad_campaignid=11612151501&amp;gbraid=0AAAAAD_uetMWPvmgHv3q_pW1Ap2XPjNcU&amp;gclid=CjwKCAjwxeHWBhBPEiwAiqtQ-fXMrRlgI_ldfpzj6iy0tx9E9ZY5jWXLAkurdtsnGW43uC5BHwLfohoCeCEQAvD_BwE</t>
+  </si>
+  <si>
+    <t>3m double sided tape</t>
+  </si>
+  <si>
+    <t>6 ft</t>
+  </si>
+  <si>
+    <t>adhesive velcro singe sided</t>
+  </si>
+  <si>
+    <t>5 ft</t>
+  </si>
+  <si>
+    <t>https://www.mcmaster.com/94985K27/</t>
+  </si>
+  <si>
+    <t>Duct tape</t>
+  </si>
+  <si>
+    <t>10 ft</t>
+  </si>
+  <si>
+    <t>https://www.homedepot.com/p/Duck-Pro-1-88-in-x-60-yds-Silver-All-Purpose-Duct-Tape-242760/309334754</t>
+  </si>
+  <si>
+    <t>https://www.homedepot.com/p/GrillPro-100-Piece-12-in-Bamboo-Skewers-11070/322906473</t>
   </si>
 </sst>
 </file>
@@ -810,19 +822,19 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="A1:B1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="16.5546875" customWidth="1"/>
+    <col min="2" max="2" width="16.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
       <c r="B1" s="4">
         <f>SUM('Per Assembly Cost --&gt;'!B:B)</f>
-        <v>361.51941778975743</v>
+        <v>367.17941778975739</v>
       </c>
     </row>
   </sheetData>
@@ -845,54 +857,54 @@
     <tabColor theme="1"/>
   </sheetPr>
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.33203125" customWidth="1"/>
-    <col min="2" max="2" width="22.88671875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="23.28515625" customWidth="1"/>
+    <col min="2" max="2" width="22.85546875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B2" s="5">
         <f>SUM('Avionics BOM'!D:D)</f>
         <v>14.695417789757411</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B3" s="1">
         <f>SUM('Structures BOM'!D:D)</f>
-        <v>152.80300000000003</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+        <v>157.93299999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B4" s="1">
         <f>SUM('Mechanisms BOM'!D:D)</f>
         <v>53.330999999999996</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B5" s="1">
         <f>SUM('Propulsion BOM'!D:D)</f>
-        <v>140.69</v>
+        <v>141.22</v>
       </c>
     </row>
   </sheetData>
@@ -906,22 +918,22 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.33203125" customWidth="1"/>
-    <col min="2" max="2" width="10.44140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="9.109375" style="1"/>
-    <col min="4" max="4" width="10.33203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.109375" style="2"/>
+    <col min="1" max="1" width="30.28515625" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="9.140625" style="1"/>
+    <col min="4" max="4" width="10.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>3</v>
@@ -930,18 +942,18 @@
         <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C2" s="1">
         <v>4</v>
@@ -950,18 +962,18 @@
         <v>7.16</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C3" s="1">
         <v>1</v>
@@ -970,18 +982,18 @@
         <v>1.59</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C4" s="1">
         <v>3</v>
@@ -991,18 +1003,18 @@
         <v>2.9699999999999998</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C5" s="1">
         <v>20</v>
@@ -1012,18 +1024,18 @@
         <v>2.6954177897574123</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C6" s="1">
         <v>1</v>
@@ -1032,10 +1044,10 @@
         <v>0.28000000000000003</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1061,22 +1073,22 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:N23"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.109375" style="1"/>
-    <col min="5" max="5" width="11.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.109375" style="2"/>
+    <col min="1" max="1" width="37.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" style="1"/>
+    <col min="5" max="5" width="11.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>3</v>
@@ -1085,18 +1097,18 @@
         <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C2" s="1">
         <v>1</v>
@@ -1105,18 +1117,18 @@
         <v>26.26</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C3" s="1">
         <v>1</v>
@@ -1126,18 +1138,18 @@
         <v>27.8</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C4" s="1">
         <v>5</v>
@@ -1146,18 +1158,18 @@
         <v>2.97</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C5" s="1">
         <v>25</v>
@@ -1166,18 +1178,18 @@
         <v>4.5999999999999996</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>1</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C6" s="1">
         <v>25</v>
@@ -1186,18 +1198,18 @@
         <v>5.55</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C7" s="1">
         <v>100</v>
@@ -1206,18 +1218,18 @@
         <v>3.93</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C8" s="1">
         <v>25</v>
@@ -1226,18 +1238,18 @@
         <v>7.14</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C9" s="1">
         <v>1</v>
@@ -1246,18 +1258,18 @@
         <v>24.6</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C10" s="1">
         <v>1</v>
@@ -1266,18 +1278,18 @@
         <v>14.27</v>
       </c>
       <c r="E10" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>60</v>
       </c>
-      <c r="F10" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>64</v>
-      </c>
       <c r="B11" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C11" s="1">
         <v>1</v>
@@ -1286,63 +1298,63 @@
         <v>3.94</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D12" s="5">
         <f>4.98/8*6</f>
         <v>3.7350000000000003</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>72</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>76</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>80</v>
       </c>
       <c r="D13" s="5">
         <f>9.98*0.6</f>
         <v>5.9880000000000004</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>79</v>
+        <v>55</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>75</v>
       </c>
       <c r="N13" s="8" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C14" s="1">
         <v>4</v>
@@ -1352,38 +1364,38 @@
         <v>9.84</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D15" s="1">
         <v>4.07</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C16" s="1">
         <v>1</v>
@@ -1392,18 +1404,18 @@
         <v>1.0900000000000001</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C17" s="1">
         <v>1</v>
@@ -1412,41 +1424,39 @@
         <v>0.06</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C18" s="1">
         <v>1</v>
       </c>
       <c r="D18" s="1">
-        <v>0.91</v>
+        <v>0.67</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="N18" s="8" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+      <c r="N18" s="8"/>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C19" s="1">
         <v>4</v>
@@ -1455,46 +1465,95 @@
         <v>0.05</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C20" s="1">
-        <v>3</v>
+        <v>26</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="D20" s="1">
-        <v>6</v>
+        <v>0.51</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="N20" s="8" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="N21" s="8" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="N22" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="F20" s="3" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="N23" s="8" t="s">
-        <v>88</v>
-      </c>
+      <c r="N20" s="8"/>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>90</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="D21" s="1">
+        <v>7.76</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="N21" s="8"/>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>93</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="D22" s="1">
+        <v>0.39</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="N22" s="8"/>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C23" s="1">
+        <v>100</v>
+      </c>
+      <c r="D23" s="1">
+        <v>2.71</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="N23" s="8"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="E1:E1048576">
@@ -1520,6 +1579,11 @@
     <hyperlink ref="F11" r:id="rId15" xr:uid="{9B3802E2-0DAA-4495-8E7B-C8A9F6A2FFA8}"/>
     <hyperlink ref="F19" r:id="rId16" xr:uid="{8B7798E1-B9EF-4C27-8F45-57F8754CF6C6}"/>
     <hyperlink ref="F12" r:id="rId17" xr:uid="{DAC881B0-F10F-4F69-8986-0AAA523A24EF}"/>
+    <hyperlink ref="F21" r:id="rId18" xr:uid="{B1936492-E69E-4FC0-9317-A51FD4D180C9}"/>
+    <hyperlink ref="F20" r:id="rId19" display="https://www.uline.com/Product/Detail/S-24954/3M-Double-Sided-Tape/3M-GPT-020-Double-Coated-Tape-1-2-x-55-yds?pricode=WB2129&amp;gadtype=pla&amp;id=S-24954&amp;ad_group_id=145971513970&amp;gad_source=1&amp;gad_campaignid=11612151501&amp;gbraid=0AAAAAD_uetMWPvmgHv3q_pW1Ap2XPjNcU&amp;gclid=CjwKCAjwxeHWBhBPEiwAiqtQ-fXMrRlgI_ldfpzj6iy0tx9E9ZY5jWXLAkurdtsnGW43uC5BHwLfohoCeCEQAvD_BwE" xr:uid="{5269E7F4-3C12-41E9-B94C-7D7110BCCB5B}"/>
+    <hyperlink ref="F13" r:id="rId20" xr:uid="{02A4D3AB-EDC0-4B65-841E-3298AA137928}"/>
+    <hyperlink ref="F22" r:id="rId21" xr:uid="{14143E63-1487-40FC-AEB3-356D1822FE75}"/>
+    <hyperlink ref="F23" r:id="rId22" xr:uid="{B7AFD8AB-FA10-4D01-851E-CFAF953BAB8E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1531,22 +1595,22 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:F10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.88671875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="9.109375" style="1"/>
-    <col min="4" max="4" width="10.6640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.109375" style="2"/>
+    <col min="1" max="1" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="9.140625" style="1"/>
+    <col min="4" max="4" width="10.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>3</v>
@@ -1555,18 +1619,18 @@
         <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C2" s="1">
         <v>4</v>
@@ -1575,18 +1639,18 @@
         <v>13.88</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C3" s="1">
         <v>2</v>
@@ -1595,18 +1659,18 @@
         <v>0.11</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C4" s="1">
         <v>4</v>
@@ -1615,18 +1679,18 @@
         <v>2.99</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C5" s="1">
         <v>4</v>
@@ -1635,18 +1699,18 @@
         <v>6.2759999999999998</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C6" s="1">
         <v>1</v>
@@ -1655,18 +1719,18 @@
         <v>14.99</v>
       </c>
       <c r="E6" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C7" s="1">
         <v>2</v>
@@ -1676,18 +1740,18 @@
         <v>5.9950000000000001</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C8" s="1">
         <v>1</v>
@@ -1696,18 +1760,18 @@
         <v>8.9700000000000006</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C9" s="1">
         <v>20</v>
@@ -1716,15 +1780,15 @@
         <v>0.12</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="F10" s="9" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -1750,21 +1814,21 @@
     <tabColor theme="0"/>
   </sheetPr>
   <dimension ref="A1:M5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.5546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="12.88671875" style="1" customWidth="1"/>
-    <col min="4" max="5" width="12.109375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="9.109375" style="2"/>
+    <col min="2" max="2" width="11.5703125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="12.85546875" style="1" customWidth="1"/>
+    <col min="4" max="5" width="12.140625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>3</v>
@@ -1773,41 +1837,39 @@
         <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>82</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C2" s="1">
         <v>1</v>
       </c>
       <c r="D2" s="1">
-        <v>3.64</v>
+        <v>4.17</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="M2" s="8" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+        <v>86</v>
+      </c>
+      <c r="M2" s="8"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>83</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C3" s="1">
         <v>1</v>
@@ -1816,21 +1878,19 @@
         <v>57.99</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="M3" s="8" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+        <v>84</v>
+      </c>
+      <c r="M3" s="8"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C4" s="1">
         <v>1</v>
@@ -1839,18 +1899,18 @@
         <v>38.49</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C5" s="1">
         <v>1</v>
@@ -1859,10 +1919,10 @@
         <v>40.57</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -1882,12 +1942,11 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="c440327c-db0c-40f7-973b-7bc2ae283ce2" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2116,17 +2175,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="c440327c-db0c-40f7-973b-7bc2ae283ce2" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{140E0E22-42B5-4B4A-934D-04548B25B00B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F120B44-02FC-4D2A-B0A5-AADC531A6E78}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="c440327c-db0c-40f7-973b-7bc2ae283ce2"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="3bf09d50-f695-4e18-a2ec-955b0ff6d5dc"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2151,18 +2220,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F120B44-02FC-4D2A-B0A5-AADC531A6E78}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{140E0E22-42B5-4B4A-934D-04548B25B00B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="c440327c-db0c-40f7-973b-7bc2ae283ce2"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="3bf09d50-f695-4e18-a2ec-955b0ff6d5dc"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>